<commit_message>
fix(psicosocial): validate virtual birth dates in template
</commit_message>
<xml_diff>
--- a/public/templates/plantilla_carga_virtual_psicosocial.xlsx
+++ b/public/templates/plantilla_carga_virtual_psicosocial.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Carga virtual" sheetId="1" r:id="R14e81960426743df"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="2" r:id="Rf2a742adef2842b7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Carga virtual" sheetId="1" r:id="R5f6028f57f704afd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="2" r:id="R6fc11c1e895648b2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -7354,9 +7354,13 @@
       <x:c r="E1001" s="11"/>
     </x:row>
   </x:sheetData>
-  <x:dataValidations count="1">
+  <x:dataValidations count="2">
     <x:dataValidation type="list" sqref="C2:C1001">
       <x:formula1>"CC,CE,TI,PA,PEP,PPT"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="date" errorStyle="stop" operator="between" showInputMessage="1" showErrorMessage="1" errorTitle="Fecha de nacimiento inválida" error="Usa una fecha entre 1900-01-01 y ayer. Verifica día y mes antes de guardar." promptTitle="Fecha de nacimiento" prompt="Usa AAAA-MM-DD y verifica el valor mostrado por Excel." sqref="E2:E1001">
+      <x:formula1>DATE(1900,1,1)</x:formula1>
+      <x:formula2>TODAY()-1</x:formula2>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -7422,12 +7426,12 @@
         <x:v>Conserva letras, ceros iniciales o guiones cuando correspondan.</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="15" hidden="0" customHeight="1">
+    <x:row r="9" ht="24" hidden="0" customHeight="1">
       <x:c r="A9" s="18" t="str">
         <x:v>Fecha de nacimiento</x:v>
       </x:c>
       <x:c r="B9" s="18" t="str">
-        <x:v>Usa una fecha válida en formato AAAA-MM-DD.</x:v>
+        <x:v>Usa una fecha real de Excel o AAAA-MM-DD. Verifica el valor mostrado; los textos ambiguos serán rechazados por ABRIL360.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">

</xml_diff>

<commit_message>
fix(psicosocial): unify virtual bulk assignment flow
</commit_message>
<xml_diff>
--- a/public/templates/plantilla_carga_virtual_psicosocial.xlsx
+++ b/public/templates/plantilla_carga_virtual_psicosocial.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Carga virtual" sheetId="1" r:id="R5f6028f57f704afd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="2" r:id="R6fc11c1e895648b2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Carga virtual" sheetId="1" r:id="Red6f1feabede43fa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="2" r:id="R70feb406a13046f2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -41,7 +41,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="3">
+  <x:fills count="4">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -53,8 +53,13 @@
         <x:fgColor rgb="FF0C162C"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0C162C"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="3">
+  <x:borders count="4">
     <x:border/>
     <x:border>
       <x:left style="thin">
@@ -75,11 +80,25 @@
         <x:color rgb="FF00D4B8"/>
       </x:bottom>
     </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD6E2E0"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFD6E2E0"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD6E2E0"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD6E2E0"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="20">
+  <x:cellXfs count="29">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -123,6 +142,27 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -334,6 +374,7 @@
     <x:col min="3" max="3" width="21" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="23" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="23" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="16" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="32" customHeight="1">
@@ -352,6 +393,9 @@
       <x:c r="E1" s="6" t="str">
         <x:v>Fecha de nacimiento</x:v>
       </x:c>
+      <x:c r="F1" s="28" t="str">
+        <x:v>Formulario</x:v>
+      </x:c>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="9"/>
@@ -7354,13 +7398,16 @@
       <x:c r="E1001" s="11"/>
     </x:row>
   </x:sheetData>
-  <x:dataValidations count="2">
+  <x:dataValidations count="3">
     <x:dataValidation type="list" sqref="C2:C1001">
       <x:formula1>"CC,CE,TI,PA,PEP,PPT"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="date" errorStyle="stop" operator="between" showInputMessage="1" showErrorMessage="1" errorTitle="Fecha de nacimiento inválida" error="Usa una fecha entre 1900-01-01 y ayer. Verifica día y mes antes de guardar." promptTitle="Fecha de nacimiento" prompt="Usa AAAA-MM-DD y verifica el valor mostrado por Excel." sqref="E2:E1001">
       <x:formula1>DATE(1900,1,1)</x:formula1>
       <x:formula2>TODAY()-1</x:formula2>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="F2:F1001">
+      <x:formula1>"A,B"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -7395,59 +7442,67 @@
       <x:c r="E3" s="14"/>
     </x:row>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
-      <x:c r="A5" s="19" t="str">
+      <x:c r="A5" s="6" t="str">
         <x:v>Regla</x:v>
       </x:c>
-      <x:c r="B5" s="19" t="str">
+      <x:c r="B5" s="6" t="str">
         <x:v>Descripción</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
-      <x:c r="A6" s="18" t="str">
+      <x:c r="A6" s="21" t="str">
         <x:v>Datos obligatorios</x:v>
       </x:c>
-      <x:c r="B6" s="18" t="str">
-        <x:v>Completa los cinco campos de cada colaborador. No dejes celdas vacías.</x:v>
+      <x:c r="B6" s="21" t="str">
+        <x:v>Completa los seis campos de cada colaborador. No dejes celdas vacías.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
-      <x:c r="A7" s="18" t="str">
+      <x:c r="A7" s="21" t="str">
         <x:v>Tipo de documento</x:v>
       </x:c>
-      <x:c r="B7" s="18" t="str">
-        <x:v>Usa únicamente CC, CE, TI, PA, PEP o PPT.</x:v>
+      <x:c r="B7" s="21" t="str">
+        <x:v>Usa CC, CE, TI, PA, PEP o PPT.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
-      <x:c r="A8" s="18" t="str">
+      <x:c r="A8" s="21" t="str">
         <x:v>Número de documento</x:v>
       </x:c>
-      <x:c r="B8" s="18" t="str">
+      <x:c r="B8" s="21" t="str">
         <x:v>Conserva letras, ceros iniciales o guiones cuando correspondan.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="24" hidden="0" customHeight="1">
-      <x:c r="A9" s="18" t="str">
+      <x:c r="A9" s="21" t="str">
         <x:v>Fecha de nacimiento</x:v>
       </x:c>
-      <x:c r="B9" s="18" t="str">
+      <x:c r="B9" s="21" t="str">
         <x:v>Usa una fecha real de Excel o AAAA-MM-DD. Verifica el valor mostrado; los textos ambiguos serán rechazados por ABRIL360.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
-      <x:c r="A10" s="18" t="str">
+      <x:c r="A10" s="21" t="str">
+        <x:v>Formulario</x:v>
+      </x:c>
+      <x:c r="B10" s="21" t="str">
+        <x:v>Selecciona A o B según el formulario asignado al colaborador.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="24" hidden="0" customHeight="1">
+      <x:c r="A11" s="21" t="str">
         <x:v>Una persona por fila</x:v>
       </x:c>
-      <x:c r="B10" s="18" t="str">
-        <x:v>No repitas la combinación de tipo y número de documento.</x:v>
+      <x:c r="B11" s="21" t="str">
+        <x:v>No repitas documentos dentro del archivo. El máximo es 1.000 colaboradores.</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="24" hidden="0" customHeight="1">
-      <x:c r="A11" s="18" t="str">
+    <x:row r="12">
+      <x:c r="A12" s="22" t="str">
         <x:v>Certificación</x:v>
       </x:c>
-      <x:c r="B11" s="18" t="str">
-        <x:v>Antes de importar, el profesional debe certificar que los datos son correctos porque se usarán para verificar el acceso.</x:v>
+      <x:c r="B12" s="22" t="str">
+        <x:v>Antes de importar deberás certificar que los datos y el formulario son correctos.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>